<commit_message>
Route Slack digest to sales sheet
</commit_message>
<xml_diff>
--- a/docs/templates/company_detector_sales_sheet_template.xlsx
+++ b/docs/templates/company_detector_sales_sheet_template.xlsx
@@ -354,7 +354,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
+    <row r="6" ht="74" customHeight="1">
       <c r="A6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">21 Mei 2026, 09:00 WIB</t>
@@ -392,9 +392,23 @@
       </c>
       <c r="H6" s="0"/>
       <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="K6" s="0"/>
-      <c r="L6" s="0"/>
+      <c r="J6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tokopedia: https://www.tokopedia.com/falasik</t>
+        </is>
+      </c>
+      <c r="K6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instagram: https://instagram.com/falasik
+TikTok: https://tiktok.com/@falasik
+LinkedIn: https://au.linkedin.com/in/falasik</t>
+        </is>
+      </c>
+      <c r="L6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://falasik.com</t>
+        </is>
+      </c>
       <c r="M6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Register platform</t>

</xml_diff>